<commit_message>
session 27: python patterns
</commit_message>
<xml_diff>
--- a/Daily_Report.xlsx
+++ b/Daily_Report.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data_Science\01_Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{12E4199D-3C6A-4CA2-BDF2-35E5F59C5124}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AB3616CD-C46D-4AA1-A883-8FA20992989E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="126" uniqueCount="111">
   <si>
     <t>Date</t>
   </si>
@@ -498,6 +498,12 @@
   </si>
   <si>
     <t xml:space="preserve">Functions: title, subheader, text, write, success, error, button, radio, selectbox, slider, date_input, text_input, number_input, image, columns, file_uploader, dataframe, </t>
+  </si>
+  <si>
+    <t>Python Patterns</t>
+  </si>
+  <si>
+    <t>right angle triangle pattern, inverted right angle triangle pattern, pyramid pattern, inverted pyramid, diamond, hallow sqaure, full square, right angle (number), inverted right angle traingle (number), floyds tiangle, hallow right angle trianlge, hallow pyramid, hallow diamon, haloow diamon (number), butterfly, hallow number pyrrmid, full star pyramind, inverted full star pyramid, lef aligned pyramind, right alinged pyramind.</t>
   </si>
 </sst>
 </file>
@@ -939,7 +945,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="17.399999999999999" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.44140625" style="13" bestFit="1" customWidth="1"/>
@@ -1124,7 +1130,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="12" spans="1:7" ht="156.6" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:7" ht="139.19999999999999" x14ac:dyDescent="0.25">
       <c r="A12" s="13">
         <v>11</v>
       </c>
@@ -1166,7 +1172,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="156.6" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:7" ht="139.19999999999999" x14ac:dyDescent="0.25">
       <c r="A15" s="13">
         <v>14</v>
       </c>
@@ -1346,6 +1352,20 @@
       </c>
       <c r="D27" s="12" t="s">
         <v>108</v>
+      </c>
+    </row>
+    <row r="28" spans="1:4" ht="87" x14ac:dyDescent="0.25">
+      <c r="A28" s="13">
+        <v>27</v>
+      </c>
+      <c r="B28" s="14">
+        <v>46119</v>
+      </c>
+      <c r="C28" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="D28" s="12" t="s">
+        <v>110</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
session 39: data visualization using plots
</commit_message>
<xml_diff>
--- a/Daily_Report.xlsx
+++ b/Daily_Report.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Data_Science\01_Practice\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0D4303BC-AF66-4D46-85E9-FA3C532B2B18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F81B12C3-F4B7-41ED-B773-3D59EC651390}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="75" uniqueCount="74">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="85">
   <si>
     <t>Date</t>
   </si>
@@ -349,6 +349,39 @@
   </si>
   <si>
     <t>Array creation, slicing, axis-wise aggregations (sum/min/max/mean), cumsum, dot product, np.vectorize, np.save/load, image as array, CSV loading, feature extraction with .apply(), regex on columns, EDA (describe/info/value_counts), conditional filtering, string cleaning</t>
+  </si>
+  <si>
+    <t>Data Visualization-2</t>
+  </si>
+  <si>
+    <t>Data Visualization-1</t>
+  </si>
+  <si>
+    <t>seaborn, matplotlib, histplot, kdeplot, countplot, barplot</t>
+  </si>
+  <si>
+    <t>boxplot, violinplot, stripplot, scatterplot, regplot, heatmap, pairplot, FacetGrid</t>
+  </si>
+  <si>
+    <t>SQL-1</t>
+  </si>
+  <si>
+    <t>SQL-2</t>
+  </si>
+  <si>
+    <t>MYSql shell, workbernch into, show db, create db, create table, insert record, insert multiple records, see the tables, see the specific table content, see the specific attributes</t>
+  </si>
+  <si>
+    <t>sum, average, count, asc desc, wild card, like %, joins: inner; outer; cross; left; right</t>
+  </si>
+  <si>
+    <t>EDA-Pro (Project)</t>
+  </si>
+  <si>
+    <t>pandas, numpy, matplotlib, streamlit</t>
+  </si>
+  <si>
+    <t>weasyPrint, pytest, type hints, google style docstrings, OOP, git</t>
   </si>
 </sst>
 </file>
@@ -749,7 +782,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:G34"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="18" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="13.44140625" style="6" bestFit="1" customWidth="1"/>
@@ -1256,6 +1289,87 @@
         <v>71</v>
       </c>
     </row>
+    <row r="35" spans="1:4" ht="36" x14ac:dyDescent="0.25">
+      <c r="A35" s="6">
+        <v>34</v>
+      </c>
+      <c r="B35" s="7">
+        <v>46128</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D35" s="5" t="s">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="36" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A36" s="6">
+        <v>35</v>
+      </c>
+      <c r="B36" s="7">
+        <v>46129</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>79</v>
+      </c>
+      <c r="D36" s="6" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="37" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A37" s="6">
+        <v>36</v>
+      </c>
+      <c r="B37" s="7">
+        <v>46132</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>82</v>
+      </c>
+      <c r="D37" s="6" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="38" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A38" s="6">
+        <v>37</v>
+      </c>
+      <c r="B38" s="7">
+        <v>46133</v>
+      </c>
+      <c r="D38" s="6" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="39" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A39" s="6">
+        <v>38</v>
+      </c>
+      <c r="B39" s="7">
+        <v>46134</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D39" s="6" t="s">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="40" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A40" s="6">
+        <v>39</v>
+      </c>
+      <c r="B40" s="7">
+        <v>46135</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>74</v>
+      </c>
+      <c r="D40" s="6" t="s">
+        <v>77</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>